<commit_message>
Water billing dashboard modification
</commit_message>
<xml_diff>
--- a/media/hr_documents/CUSTOMERS.xlsx
+++ b/media/hr_documents/CUSTOMERS.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\VERSATEC DOCUMENTS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\VMS\vicms\media\hr_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD2C8A74-6552-4F4C-BB6B-4A8405E43E0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFAF4DD1-D7BE-4517-AA36-9C35252495CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{8F300229-77B4-44C2-B17A-36348983AA07}"/>
   </bookViews>
@@ -1260,7 +1260,7 @@
     <t>GARSUTA, JUVY</t>
   </si>
   <si>
-    <t xml:space="preserve">  </t>
+    <t>NATIVIDAD ARGUELLES</t>
   </si>
 </sst>
 </file>
@@ -1287,6 +1287,7 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -7153,7 +7154,7 @@
       <c r="B331" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C331" s="4" t="s">
+      <c r="C331" s="2" t="s">
         <v>408</v>
       </c>
       <c r="D331" s="5">

</xml_diff>